<commit_message>
test data files data driven testing
</commit_message>
<xml_diff>
--- a/seleniumTesting/src/test/resources/testData/data.xlsx
+++ b/seleniumTesting/src/test/resources/testData/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\automation\selenium automation\seleniumAutomation\seleniumTesting\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{194AFE90-BEF7-4139-9C51-A8A127981405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB211E63-2457-42BB-B899-90AB011149C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{784EB5F0-9922-4251-8F18-0192C8ED9C99}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -123,7 +123,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>

</xml_diff>